<commit_message>
Greif funcional e criado filtro de exclusão pra cpf e data_inicio nulos
</commit_message>
<xml_diff>
--- a/aa.xlsx
+++ b/aa.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y5"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GREIF ARATU</t>
+          <t>GREIF PARANA/ARAUCARIA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -573,17 +573,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>20415</t>
+          <t>20423</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LUCIANO DA SILVA DA CRUZ</t>
+          <t>BRUNO NASCIMENTO JACONELLI</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>303245</t>
+          <t>2106024</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -620,43 +620,43 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>LUCIANO DA SILVA DA CRUZ</t>
+          <t>BRUNO NASCIMENTO JACONELLI</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>809.795.305-63</t>
+          <t>427.771.148-03</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
-        <v>45905</v>
+        <v>45903</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hapvida </t>
+          <t xml:space="preserve">Policlinica capao raso </t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>G-40</t>
+          <t>G43</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Miriam Sepulveda</t>
+          <t xml:space="preserve">Marcio Duarte Coutinho </t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>3784</v>
+        <v>23104</v>
       </c>
     </row>
     <row r="3">
@@ -665,7 +665,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GREIF PARANA/ARAUCARIA</t>
+          <t>Greif SP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -678,24 +678,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20413</t>
+          <t>20439</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LUCINEIA MARIA DE JESUS SOUZA</t>
+          <t>DEUSEIR WILLIAN PEREIRA DE BARROS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2105782</t>
+          <t>141479</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>45905</v>
+        <v>45908</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>45910</v>
+        <v>45913</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -725,230 +725,24 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>LUCINEIA MARIA DE JESUS SOUZA</t>
+          <t>DEUSEIR WILLIAN PEREIRA DE BARROS</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>023.512.739-66</t>
+          <t>317.399.508-28</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" s="2" t="n">
-        <v>45902</v>
-      </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>0</v>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Ima</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Josiane malc barbosa</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="Y3" t="n">
-        <v>13065</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GREIF ESTEIO</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>20412</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>MARCIO ROGERIO TAVARES</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>602493</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>45905</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>45910</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Expert</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Atestado médico</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Envio de Atestado Médico</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Atestado Médico</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Expert</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>MARCIO ROGERIO TAVARES</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>749.895.530-04</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>GREIF PARANA/ARAUCARIA</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Pendente</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>20418</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>ANDREIA CRISTIANE DE ANDRADE SILVA</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2105823</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>45905</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>45910</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Expert</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Atestado médico</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Envio de Atestado Médico</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Atestado Médico</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Expert</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>ANDREIA CRISTIANE DE ANDRADE SILVA</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>052.048.979-92</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" s="2" t="n">
-        <v>45904</v>
-      </c>
-      <c r="T5" t="n">
-        <v>1</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Cirurgia Plástica Doutor Alexandre Wood Branco</t>
-        </is>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>ALEXANDRE WOOD BRANCO</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>CRM 15517</t>
-        </is>
-      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>